<commit_message>
Add client-ready rental shortlist page; note Rio Vista feeder bus
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015SAzJzLnM21KpQ1dEcchKU
</commit_message>
<xml_diff>
--- a/output/rental_search_revised_2026-09-30.xlsx
+++ b/output/rental_search_revised_2026-09-30.xlsx
@@ -575,7 +575,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Hougang/Buangkok NEL (walk or feeder bus, confirm)</t>
+          <t>Hougang/Buangkok NEL (feeder bus)</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Hougang/Buangkok NEL</t>
+          <t>Hougang/Buangkok NEL (feeder bus)</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -675,7 +675,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hougang/Buangkok NEL</t>
+          <t>Hougang/Buangkok NEL (feeder bus)</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Hougang/Buangkok NEL</t>
+          <t>Hougang/Buangkok NEL (feeder bus)</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">

</xml_diff>